<commit_message>
Bugfix A14, A15 pin assign
A14, A15 のピンアサインがあべこべになっていたバグを修正
</commit_message>
<xml_diff>
--- a/doc/FPGA_MSXtR_Stack_TangFPGA_pin.xlsx
+++ b/doc/FPGA_MSXtR_Stack_TangFPGA_pin.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hra\Documents\github\HRA_product\FPGA_MSXtR\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B20DF5-19D9-41ED-9307-49340BE8DEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659AC1CF-8DC5-47F3-8721-E29C64D246CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4363,8 +4363,8 @@
       <c r="W26" s="48">
         <v>106</v>
       </c>
-      <c r="X26" s="1" t="s">
-        <v>286</v>
+      <c r="X26" s="29" t="s">
+        <v>290</v>
       </c>
       <c r="Y26" s="1">
         <v>7</v>
@@ -4427,8 +4427,8 @@
       <c r="W27" s="48">
         <v>108</v>
       </c>
-      <c r="X27" s="1" t="s">
-        <v>290</v>
+      <c r="X27" s="29" t="s">
+        <v>286</v>
       </c>
       <c r="Y27" s="1">
         <v>7</v>

</xml_diff>